<commit_message>
Race tab container added, working on the stats UI
</commit_message>
<xml_diff>
--- a/GameData/RaceResources/races.xlsx
+++ b/GameData/RaceResources/races.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C695203-C694-42D6-A56B-3E30C03E41DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{737F6D37-5F25-45F6-907D-CF8F13FBA5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="106">
   <si>
     <t>race_id</t>
   </si>
@@ -303,13 +303,52 @@
     <t>"nightvision,elegance,fae_descent,pretty"</t>
   </si>
   <si>
-    <t>"imposed_element_earth,big_bellied"</t>
-  </si>
-  <si>
     <t>"imposed_element_air"</t>
   </si>
   <si>
     <t>"imposed_element_fire,short_breath"</t>
+  </si>
+  <si>
+    <t>"imposed_element_earth,big_bellied,homely"</t>
+  </si>
+  <si>
+    <t>txtheight</t>
+  </si>
+  <si>
+    <t>"1m50 to 2m"</t>
+  </si>
+  <si>
+    <t>"1m70 to 2m20"</t>
+  </si>
+  <si>
+    <t>"1m10 to 1m50"</t>
+  </si>
+  <si>
+    <t>"2m to 2m50"</t>
+  </si>
+  <si>
+    <t>"1m80 to 2m30"</t>
+  </si>
+  <si>
+    <t>"1m40 to 1m90"</t>
+  </si>
+  <si>
+    <t>"1m50 to 2m for women, 1m90 to 2m40 for men"</t>
+  </si>
+  <si>
+    <t>"1m60 to 2m10"</t>
+  </si>
+  <si>
+    <t>"80 cm to 1m20"</t>
+  </si>
+  <si>
+    <t>"20 cm to 35 cm"</t>
+  </si>
+  <si>
+    <t>"3m plus 50cm per level"</t>
+  </si>
+  <si>
+    <t>"1m20 to 2m50"</t>
   </si>
 </sst>
 </file>
@@ -639,17 +678,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AN14"/>
+  <dimension ref="A1:AO14"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="14.77734375" customWidth="1"/>
-    <col min="6" max="6" width="13.77734375" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" customWidth="1"/>
-    <col min="8" max="8" width="11.5546875" customWidth="1"/>
-    <col min="39" max="39" width="37.77734375" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.77734375" customWidth="1"/>
+    <col min="8" max="8" width="15.44140625" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" customWidth="1"/>
+    <col min="40" max="40" width="37.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:41" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -660,118 +699,121 @@
         <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -781,32 +823,35 @@
       <c r="C2" t="s">
         <v>86</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2">
         <v>2</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
-      <c r="G2" s="2">
-        <v>0</v>
-      </c>
-      <c r="H2">
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
         <v>0</v>
       </c>
       <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
         <v>100</v>
       </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="AM2" t="s">
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -816,47 +861,50 @@
       <c r="C3" t="s">
         <v>85</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3">
         <v>2</v>
       </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
       <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3" s="2">
-        <v>0</v>
-      </c>
-      <c r="H3">
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
         <v>0</v>
       </c>
       <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
         <v>200</v>
       </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
       <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
         <v>2</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>2</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>-1</v>
       </c>
-      <c r="AA3">
+      <c r="AB3">
         <v>10</v>
       </c>
-      <c r="AH3">
+      <c r="AI3">
         <v>10</v>
       </c>
-      <c r="AM3" t="s">
+      <c r="AN3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -866,50 +914,53 @@
       <c r="C4" t="s">
         <v>87</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4">
         <v>1.5</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
       <c r="F4">
         <v>0</v>
       </c>
-      <c r="G4" s="2">
-        <v>0</v>
-      </c>
-      <c r="H4">
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
         <v>0</v>
       </c>
       <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
         <v>80</v>
       </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="L4">
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>-2</v>
-      </c>
-      <c r="O4">
-        <v>2</v>
       </c>
       <c r="P4">
         <v>2</v>
       </c>
-      <c r="V4">
+      <c r="Q4">
+        <v>2</v>
+      </c>
+      <c r="W4">
         <v>15</v>
       </c>
-      <c r="AG4">
+      <c r="AH4">
         <v>10</v>
       </c>
-      <c r="AM4" t="s">
+      <c r="AN4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -919,88 +970,91 @@
       <c r="C5" t="s">
         <v>88</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E5">
         <v>2.5</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
       <c r="F5">
         <v>0</v>
       </c>
-      <c r="G5" s="2">
-        <v>0</v>
-      </c>
-      <c r="H5">
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
         <v>0</v>
       </c>
       <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
         <v>70</v>
       </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
       <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
         <v>-2</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>-2</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>5</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>4</v>
       </c>
-      <c r="AM5" t="s">
+      <c r="AN5" t="s">
         <v>51</v>
       </c>
-      <c r="AN5" t="s">
+      <c r="AO5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>31</v>
       </c>
       <c r="B6" t="s">
         <v>71</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6">
         <v>1</v>
       </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" s="2">
-        <v>0</v>
-      </c>
-      <c r="H6">
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
         <v>0</v>
       </c>
       <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
         <v>120</v>
       </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
       <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
         <v>5</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>3</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>-3</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>-2</v>
-      </c>
-      <c r="V6">
-        <v>10</v>
       </c>
       <c r="W6">
         <v>10</v>
@@ -1008,372 +1062,399 @@
       <c r="X6">
         <v>10</v>
       </c>
-      <c r="AM6" t="s">
+      <c r="Y6">
+        <v>10</v>
+      </c>
+      <c r="AN6" t="s">
         <v>49</v>
       </c>
-      <c r="AN6" t="s">
+      <c r="AO6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
       <c r="B7" t="s">
         <v>72</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E7">
         <v>2</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
       <c r="F7">
         <v>0</v>
       </c>
-      <c r="G7" s="2">
-        <v>0</v>
-      </c>
-      <c r="H7">
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2">
         <v>0</v>
       </c>
       <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
         <v>100</v>
       </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="L7">
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="M7">
         <v>-2</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>3</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>15</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>15</v>
       </c>
-      <c r="Z7">
+      <c r="AA7">
         <v>15</v>
       </c>
-      <c r="AM7" t="s">
+      <c r="AN7" t="s">
         <v>53</v>
       </c>
-      <c r="AN7" t="s">
+      <c r="AO7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>33</v>
       </c>
       <c r="B8" t="s">
         <v>73</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8">
         <v>2.5</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
       <c r="F8">
         <v>0</v>
       </c>
-      <c r="G8" s="2">
-        <v>0</v>
-      </c>
-      <c r="H8">
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
         <v>0</v>
       </c>
       <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
         <v>60</v>
       </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
       <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
         <v>-6</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>1</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>4</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>5</v>
       </c>
-      <c r="X8">
+      <c r="Y8">
         <v>15</v>
       </c>
-      <c r="AM8" t="s">
+      <c r="AN8" t="s">
         <v>55</v>
       </c>
-      <c r="AN8" t="s">
-        <v>90</v>
+      <c r="AO8" t="s">
+        <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>34</v>
       </c>
       <c r="B9" t="s">
         <v>74</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9">
         <v>2</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
       <c r="F9">
         <v>0</v>
       </c>
-      <c r="G9" s="2">
-        <v>0</v>
-      </c>
-      <c r="H9">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
         <v>0</v>
       </c>
       <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
         <v>150</v>
       </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="M9">
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="N9">
         <v>3</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>2</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <v>15</v>
       </c>
-      <c r="AK9">
+      <c r="AL9">
         <v>10</v>
       </c>
-      <c r="AM9" t="s">
+      <c r="AN9" t="s">
         <v>56</v>
       </c>
-      <c r="AN9" t="s">
-        <v>91</v>
+      <c r="AO9" t="s">
+        <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>35</v>
       </c>
       <c r="B10" t="s">
         <v>75</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="s">
+        <v>100</v>
+      </c>
+      <c r="E10">
         <v>2</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
       <c r="F10">
         <v>0</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
         <v>1</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>0.5</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>100</v>
       </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="O10">
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>4</v>
+      </c>
+      <c r="Q10">
         <v>3</v>
       </c>
-      <c r="P10">
-        <v>2</v>
-      </c>
-      <c r="AM10" t="s">
+      <c r="AL10">
+        <v>15</v>
+      </c>
+      <c r="AN10" t="s">
         <v>57</v>
       </c>
-      <c r="AN10" t="s">
-        <v>92</v>
+      <c r="AO10" t="s">
+        <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>36</v>
       </c>
       <c r="B11" t="s">
         <v>76</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E11">
         <v>2</v>
       </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
       <c r="F11">
         <v>0</v>
       </c>
-      <c r="G11" s="2">
-        <v>0</v>
-      </c>
-      <c r="H11">
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
         <v>0</v>
       </c>
       <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
         <v>60</v>
       </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="L11">
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="M11">
         <v>3</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>2</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>1</v>
-      </c>
-      <c r="O11">
-        <v>-3</v>
       </c>
       <c r="P11">
         <v>-3</v>
       </c>
-      <c r="AM11" t="s">
+      <c r="Q11">
+        <v>-3</v>
+      </c>
+      <c r="AN11" t="s">
         <v>58</v>
       </c>
-      <c r="AN11" t="s">
+      <c r="AO11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>37</v>
       </c>
       <c r="B12" t="s">
         <v>77</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="s">
+        <v>103</v>
+      </c>
+      <c r="E12">
         <v>0.5</v>
       </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
       <c r="F12">
         <v>0</v>
       </c>
-      <c r="G12" s="2">
-        <v>0</v>
-      </c>
-      <c r="H12">
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
         <v>0</v>
       </c>
       <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
         <v>300</v>
       </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
       <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
         <v>3</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>6</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>-5</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>-3</v>
       </c>
-      <c r="AM12" t="s">
+      <c r="AN12" t="s">
         <v>60</v>
       </c>
-      <c r="AN12" t="s">
+      <c r="AO12" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>38</v>
       </c>
       <c r="B13" t="s">
         <v>78</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13">
         <v>3</v>
       </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
       <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
         <v>1</v>
       </c>
-      <c r="G13" s="2">
-        <v>0</v>
-      </c>
-      <c r="H13">
+      <c r="H13" s="2">
+        <v>0</v>
+      </c>
+      <c r="I13">
         <v>0.5</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>80</v>
       </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="AM13" t="s">
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="AN13" t="s">
         <v>62</v>
       </c>
-      <c r="AN13" t="s">
+      <c r="AO13" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>39</v>
       </c>
       <c r="B14" t="s">
         <v>79</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="s">
+        <v>105</v>
+      </c>
+      <c r="E14">
         <v>1.5</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>1</v>
       </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2">
-        <v>0</v>
-      </c>
-      <c r="H14">
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0</v>
+      </c>
+      <c r="I14">
         <v>1</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>60</v>
       </c>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="N14">
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="O14">
         <v>-2</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>-3</v>
-      </c>
-      <c r="V14">
-        <v>-10</v>
       </c>
       <c r="W14">
         <v>-10</v>
@@ -1381,10 +1462,13 @@
       <c r="X14">
         <v>-10</v>
       </c>
-      <c r="AM14" t="s">
+      <c r="Y14">
+        <v>-10</v>
+      </c>
+      <c r="AN14" t="s">
         <v>64</v>
       </c>
-      <c r="AN14" t="s">
+      <c r="AO14" t="s">
         <v>65</v>
       </c>
     </row>

</xml_diff>